<commit_message>
Update 2026 list to 45 approvals (through 2026-09-28)
- Add 12 novel approvals (Rasonque through Emcitate), FDA list current as of 09/28/2026
- Fill Pasatru application number (BLA 761508) and newly posted review (TOC) links
- Recompute 2026 TA/company analysis for 45 approvals
- Remove note about review PDFs being saved locally

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FDA_2026_Novel_Drugs_Dashboard.xlsx
+++ b/FDA_2026_Novel_Drugs_Dashboard.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1366,11 +1366,7 @@
           <t>FDA Review (TOC)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Review PDFs saved locally (ChemR, ClinPharmR, MedR, NameR, OtherR, PharmR, RiskR, AdminCorres, OEList) in C:\0_MBA\Healthcare\Baxfendy</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1897,10 +1893,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Accelerated Approval (first dual BAFF/APRIL inhibitor for IgA nephropathy). As of 2026-08-22 (46 days post-approval) only the Label and Approval Letter are posted on Drugs@FDA — no Review (TOC) package yet, longer than the typical ~30-day posting lag.</t>
+          <t>Accelerated Approval (first dual BAFF/APRIL inhibitor for IgA nephropathy). Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2013,10 +2013,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>First oral PCSK9 inhibitor approved. Type 1 NME, Priority Review. As of 2026-08-22, only the Approval Letter is posted on Drugs@FDA — Label and Review package not yet available. Listed as "MSD" (Merck's ex-US corporate name) on Drugs@FDA.</t>
+          <t>First oral PCSK9 inhibitor approved. Type 1 NME, Priority Review. Listed as "MSD" (Merck's ex-US corporate name) on Drugs@FDA. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2069,10 +2073,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Type 1 NME, Standard Review, Orphan Drug. Applicant of record on Drugs@FDA is Nuvalent (acquired by GSK; GSK led the public approval announcement). Like Idvynso, this application's label filename omits the 'Orig1' segment (220185s000lbl.pdf). No Review package posted yet as of 2026-08-22.</t>
+          <t>Type 1 NME, Standard Review, Orphan Drug. Applicant of record on Drugs@FDA is Nuvalent (acquired by GSK; GSK led the public approval announcement). Like Idvynso, this application's label filename omits the 'Orig1' segment (220185s000lbl.pdf). Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2125,10 +2133,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>First FDA-approved ophthalmic formulation of bevacizumab. Despite press coverage describing this as a 'resubmission,' Drugs@FDA shows this BLA number (761320) as ORIG-1 — a standalone application, not a later review cycle of an earlier CRL'd BLA. No Review package posted yet as of 2026-08-22.</t>
+          <t>First FDA-approved ophthalmic formulation of bevacizumab. Despite press coverage describing this as a 'resubmission,' Drugs@FDA shows this BLA number (761320) as ORIG-1 — a standalone application, not a later review cycle of an earlier CRL'd BLA. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2181,10 +2193,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>First approved norepinephrine-dopamine-serotonin reuptake inhibitor (NDSRI) for ADHD. Type 1 NME, Priority Review. No Review package posted yet as of 2026-08-22.</t>
+          <t>First approved norepinephrine-dopamine-serotonin reuptake inhibitor (NDSRI) for ADHD. Type 1 NME, Priority Review. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2237,10 +2253,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>First orexin receptor 2 (OX2R) agonist approved; internal code TAK-861. Type 1 NME, Priority Review + Orphan Drug. No Review package posted yet as of 2026-08-22 (17 days post-approval — expected).</t>
+          <t>First orexin receptor 2 (OX2R) agonist approved; internal code TAK-861. Type 1 NME, Priority Review + Orphan Drug. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2293,10 +2313,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>F18-labeled tau PET imaging agent (internal code MK-6240). Type 1 NME, Standard Review. Applicant on Drugs@FDA is Cerveau Technologies Inc, a Lantheus company. No Review package posted yet as of 2026-08-22 (9 days post-approval — expected).</t>
+          <t>F18-labeled tau PET imaging agent (internal code MK-6240). Type 1 NME, Standard Review. Applicant on Drugs@FDA is Cerveau Technologies Inc, a Lantheus company. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2349,10 +2373,14 @@
           <t>Drugs@FDA</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Accelerated Approval — first FDA-approved CELMoD (cereblon-modulating protein degrader), and the first accelerated approval in myeloma based on minimal residual disease (MRD) as an early endpoint. Type 1 NME, Priority Review + Orphan Drug. No Review package posted yet as of 2026-08-22 (9 days post-approval — expected).</t>
+          <t>Accelerated Approval — first FDA-approved CELMoD (cereblon-modulating protein degrader), and the first accelerated approval in myeloma based on minimal residual disease (MRD) as an early endpoint. Type 1 NME, Priority Review + Orphan Drug. Review (TOC) package confirmed posted as of 2026-10-04.</t>
         </is>
       </c>
     </row>
@@ -2390,21 +2418,709 @@
           <t>Regeneron</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>BLA 761508</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Original (Orig1)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Drugs@FDA (search)</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Application Number not yet indexed on Drugs@FDA as of 2026-08-22 (only 3 days post-approval) — searched by both brand name "Pasatru" and active ingredient "garetosmab", no match found under either. Not even the Label/Approval Letter are posted yet. First and only approved treatment for FOP (fibrodysplasia ossificans progressiva); first-in-class Activin A inhibitor.</t>
+          <t>UPDATED 2026-10-04: Application number now indexed on Drugs@FDA — BLA 761508, applicant Regeneron Pharmaceuticals, Orig-1, Orphan; Label, Letter and Review (TOC) all posted. First-in-class Activin A inhibitor for FOP (fibrodysplasia ossificans progressiva) — the second FOP therapy after Sohonos (palovarotene, 2023).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Rasonque</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>daraxonrasib</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>To treat metastatic pancreatic adenocarcinoma in adults who have received at least one prior systemic therapy or who are not candidates for multiagent systemic therapy</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Revolution Medicines</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NDA 220910</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>First approved RAS(ON) multi-selective inhibitor; randomized Phase 3 showed median OS 13.2 vs 6.7 months vs standard of care. Type 1 NME, Priority Review. Label and Approval Letter posted; Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Lisraya</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>brepocitinib</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>To treat dermatomyositis in adults</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Rheumatology / Immunology</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Priovant Therapeutics (Roivant)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>NDA 220106</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>TYK2/JAK1 inhibitor (listed on Drugs@FDA as brepocitinib tosylate). Type 1 NME, Priority Review. Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mimrylo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rusfertide</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>To treat erythrocytosis in adults with polycythemia vera</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Oncology / Hematology</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Takeda (Protagonist Therapeutics)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NDA 220605</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>First-in-class hepcidin mimetic peptide (listed as rusfertide acetate). Applicant of record on Drugs@FDA is Takeda; discovered by Protagonist Therapeutics. Type 1 NME, Priority Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Zanvastro</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>zilganersen</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>To treat Alexander disease in pediatric and adult patients</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Rare Disease / Neurology</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Ionis Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NDA 220210</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>FDA Review (TOC)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Antisense oligonucleotide targeting GFAP; first approved treatment for Alexander disease. Type 1 NME, Priority Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Etcamah</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>camizestrant</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>To treat hormone receptor-positive, HER2-negative, locally advanced or metastatic breast cancer upon detection of ESR1 mutation during aromatase inhibitor and CDK4/6 inhibitor therapy</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>AstraZeneca</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NDA 220359</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Oral SERD; indication tied to switching therapy when an ESR1 mutation emerges during first-line AI + CDK4/6 inhibitor treatment. Type 1 NME, Standard Review. Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Isembyld</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>apitegromab-mstn</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>To treat spinal muscular atrophy in adults and pediatric patients 2 years of age and older who are currently receiving an SMN2-targeted treatment</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Rare Disease / Neurology</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Scholar Rock</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>BLA 761463</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>First-in-class muscle-targeted anti-myostatin antibody, used as add-on to SMN2-targeted therapy. Orphan. Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Pixclara</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>floretyrosine F 18</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>To use with positron emission tomography to differentiate recurrent or progressive glioma from treatment-related change in conjunction with other diagnostic evaluations</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Diagnostic / Radiology</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Telix Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NDA 218592</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Amino-acid PET imaging agent (F-18 FET). Type 1 NME, Priority Review. Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Onswik</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>insulin efsitora alfa-gobe</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>To improve glycemic control in adults with type 2 diabetes mellitus, as an adjunct to diet and exercise</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Endocrinology / Metabolic</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Eli Lilly</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>BLA 761408</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Once-weekly basal insulin. As of 2026-10-04 only the Approval Letter is posted on Drugs@FDA (Label shown as 'not available').</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Lyrfigtu</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>lirafugratinib</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>To treat adults with previously treated unresectable, locally advanced or metastatic cholangiocarcinoma harboring a fibroblast growth factor receptor 2 gene fusion or other rearrangement</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Oncology</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Elevar Therapeutics</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NDA 220425</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Highly selective FGFR2 inhibitor (listed as lirafugratinib hydrochloride); based on single-arm Phase 2 REFOCUS (ORR 46%). Type 1 NME, Priority Review. Review package not yet posted as of 2026-10-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Juvmo</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>tavapadon</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>To treat Parkinson's disease in adults</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Neurology</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>AbbVie</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>NDA 220415</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>D1/D5 dopamine receptor partial agonist. Type 1 NME, Standard Review. As of 2026-10-04 only the Approval Letter is posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Atebrioz</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>zilurgisertib</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>To reduce the volume of total new heterotopic ossification in adults and pediatric patients 12 years and older with fibrodysplasia ossificans progressiva</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Rare Disease / Musculoskeletal</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Incyte (Mirum Pharmaceuticals)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>NDA 221198</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Oral ALK2 inhibitor; the third FOP therapy (after Sohonos 2023 and Pasatru 2026-08-19) and the first for patients as young as 12. Applicant of record on Drugs@FDA is Incyte; commercialized with Mirum. Type 1 NME, Priority Review. As of 2026-10-04 only the Approval Letter is posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Emcitate</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>tiratricol</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>To treat peripheral thyrotoxicosis in patients with MCT8 deficiency</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Rare Disease / Metabolic</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Egetis Therapeutics (Rare Thyroid Therapeutics)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>NDA 220963</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Original (Orig1)</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Drugs@FDA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Thyroid hormone analog (Triac) for MCT8 deficiency (Allan-Herndon-Dudley syndrome). Applicant on Drugs@FDA is Rare Thyroid Therapeutics International AB (an Egetis company). Label filename omits 'Orig1' (220963s000lbl.pdf). Type 1 NME, Priority Review.</t>
         </is>
       </c>
     </row>
@@ -2457,15 +3173,39 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2477,7 +3217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2486,14 +3226,14 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Content current as of: FDA's Novel Drug Approvals for 2026 page states "Content current as of: 08/19/2026". The list's last entry (Pasatru) is approved 2026-08-19, and no entries beyond that date were present when checked on 2026-08-22.</t>
+          <t>Content current as of: FDA's Novel Drug Approvals for 2026 page states "Content current as of: 09/28/2026". The list's last entry (Emcitate) is approved 2026-09-28; checked on 2026-10-04 (45 approvals).</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Application numbers were resolved via Drugs@FDA (browse-by-letter and overview.process&amp;varApplNo=) and cross-checked against web search / press releases. Rows 20 (Cypsedo), 21 (Ambelvist), and 23 (Lumvoa) — previously unconfirmed — were newly resolved in this 2026-08-22 update.</t>
+          <t>Application numbers were resolved via Drugs@FDA (browse-by-letter and overview.process&amp;varApplNo=) and cross-checked against web search / press releases. Rows 20 (Cypsedo), 21 (Ambelvist), and 23 (Lumvoa) were resolved in the 2026-08-22 update; row 33 (Pasatru, BLA 761508) was resolved in the 2026-10-04 update.</t>
         </is>
       </c>
     </row>
@@ -2507,14 +3247,14 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Submission column: "Original (Orig1)" means this was the application's first review cycle that led to approval. "Resubmission (Orig2)" means an earlier original submission was not approved and the approved application is a later review cycle. Awiqli is the only confirmed Orig2 in this list. Pasatru is marked "Unknown" because the application number itself is unconfirmed.</t>
+          <t>Submission column: "Original (Orig1)" means this was the application's first review cycle that led to approval. "Resubmission (Orig2)" means an earlier original submission was not approved and the approved application is a later review cycle. Awiqli is the only confirmed Orig2 in this list.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BLA review documents are filed under the accessdata.fda.gov /nda/ path, not /bla/ — applies to Loargys, Avlayah, Awiqli, Hepcludex, Decnupaz, Trutakna, Lytenava.</t>
+          <t>BLA review documents are filed under the accessdata.fda.gov /nda/ path, not /bla/ — applies to Loargys, Avlayah, Awiqli, Hepcludex, Decnupaz, Trutakna, Lytenava, Pasatru, Isembyld, Onswik.</t>
         </is>
       </c>
     </row>
@@ -2528,21 +3268,14 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Drugs@FDA column logic: when the Application Number is confirmed, Drugs@FDA links via event=overview.process&amp;varApplNo={number}. Only when unconfirmed (Pasatru) does it fall back to the blank search page with the drug name shown as a typing reminder.</t>
+          <t>Drugs@FDA column logic: when the Application Number is confirmed, Drugs@FDA links via event=overview.process&amp;varApplNo={number}. As of 2026-10-04 all 45 application numbers are confirmed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Review (TOC) lag: FDA review documents (Multi-Discipline/Clinical/Statistical Review etc.) typically post ~30 days after approval, after the Label and Approval Letter (which post within days). As of 2026-08-22, eight recently-approved drugs (Trutakna, Lipfendra, Jideytro, Lytenava, Simtriyo, Orzeyful, Tauklarify, Zenbexus) do not yet have a Review package posted — this is expected, not a search failure. Revtorpyk (approved 7/14) does already have its Review package posted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Baxfendy (NDA 219878) review documents are already downloaded as PDFs in C:\0_MBA\Healthcare\Baxfendy.</t>
+          <t>Review (TOC) lag: FDA review documents (Multi-Discipline/Clinical/Statistical Review etc.) typically post ~30 days after approval, after the Label and Approval Letter (which post within days). As of 2026-10-04 all approvals through 2026-08-19 have a Review package posted; of the 12 approvals since 2026-08-26, only Mimrylo and Zanvastro have one so far — this is expected, not a search failure.</t>
         </is>
       </c>
     </row>

</xml_diff>